<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-04 Le soleil de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-04.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-04.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, papa, maman, maîtresse</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut poser le soleil en papier sur le tableau. Le linge danse au jardin. Au portail, une voix trop près serre son ventre. Le soir, elle raconte, puis elle croque une pêche au vrai soleil.</t>
+          <t>Le jardin tient le linge. Sur le volet noir, un éclat de tableau tremble. Sarah veut poser le soleil, maintenant. À l'école, le rond jaune tient ; l'éclat brille. Au portail, une voix trop près : malaise. Elle veut le dire tout de suite : les mots se cognent. Elle refuse de foncer, raconte au goûter. Merci vécu. Sur le volet, l'éclat tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le linge danse sur la corde du jardin. Un torchon rouge claque un peu, tout léger. Le vent du matin est tiède. Le portillon fait un petit bruit de fer. Papa accroche une pince en bois. Maman plie une serviette encore chaude de soleil. Le torchon rouge fait comme un drapeau. Tu as senti l'herbe, Sarah ? En ce moment, Sarah sent l'herbe encore mouillée. Elle est froide, et un peu piquante. Tes chaussures restent dans l'allée, d'accord ? D'accord, maman. Sarah pose les chaussures sur les cailloux. Tes deux pieds sont sur les cailloux. Un oiseau chante dans le cerisier. Tu as entendu l'oiseau ? Oui, papa. Il est haut. À l'école, je veux poser le soleil. Le soleil en papier. Il est dans le cartable. On part. Tu dis au revoir au jardin. Au revoir, jardin. La classe sent les feutres et le papier. La maîtresse parle du temps. Aujourd'hui, il y a du soleil. Bonjour, maîtresse. Sarah écoute. Elle prend le rond jaune, tout léger. Elle pose le soleil sur le tableau. Le papier est lisse. Il tient avec une pince. Merci, Sarah. Plus tard, c'est la sortie. La cour est chaude. Des voix jouent au loin. Près du portail, une voix parle trop près. Sarah sent un malaise. Son ventre se serre. Elle reste près du groupe. Elle regarde la maîtresse. Elle se souvient du jardin. Le soir, le linge est rentré. Le jardin est calme. La porte s'ouvre. Te voilà. Tes chaussures ont un peu de poussière. Sarah pose les chaussures dans l'allée. Elle regarde le cerisier. Le ventre est encore serré.</t>
+          <t>Le jardin tient le linge comme une main ouverte. Un torchon rouge claque, puis se tait. Le vent du matin est tiède. Le portillon fait un petit bruit de fer. Papa accroche une pince en bois. Le torchon rouge fait comme un drapeau. Tu as senti l'herbe, Sarah ? Elle est froide, un peu piquante. Maman plie une serviette chaude de soleil. Les feuilles du cerisier bougent, lentes. Tu as entendu les feuilles ? Oui, papa. Elles parlent tout haut. Près du volet noir, quelque chose brille. Sur le noir lisse, un éclat de tableau tremble. Il est petit, papa. C'est le soleil sur le volet. Je veux poser le soleil, maintenant ! Celui de la classe, le rond jaune ? Oui, sur le tableau ! Le cartable attend près des chaussures. Les chaussures, dans l'allée ? Oui, maman. Sarah pose les chaussures sur les cailloux. Tes deux pieds sont sur les cailloux ? Oui. En ce moment, Sarah prend le rond jaune. Le papier est lisse, un peu chaud. Il sent le soleil, maman. On dit au revoir au jardin ? Au revoir, jardin. Le portillon cliquette derrière eux. La classe sent les feutres et le papier. Un carré de soleil glisse sur le tableau. La maîtresse parle près du noir. Bonjour les enfants. Bonjour, maîtresse. Le rond jaune va sur le tableau. Sarah pose le soleil, sans se presser. Le papier tient. Sous le rond, l'éclat de tableau brille. Il est là. Plus tard, c'est la sortie. La cour est chaude. Des voix jouent, plus loin. Près du portail, une voix parle trop près. Sarah sent un malaise. Son ventre se serre, tout petit. Elle reste près du groupe. Elle pense au jardin, au volet. Le soir, le linge est rentré. Le jardin est calme. La porte s'ouvre. Te voilà. Tes chaussures ont un peu de poussière. Sarah veut le dire, tout de suite. Papa, au portail ! Papa parle à maman, près des chaussures. Les mots de Sarah se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Sarah ? Mon ventre s'est serré. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa s'accroupit à sa hauteur. Tu as faim ? Sarah ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le linge danse sur la corde du jardin. Un torchon rouge claque un peu, tout léger. Le vent du matin est tiède. Le portillon fait un petit bruit de fer. Papa accroche une pince en bois. Maman plie une serviette encore chaude de soleil. Le torchon rouge fait comme un drapeau. Tu as senti l'herbe, Sarah ? En ce moment, Sarah sent l'herbe encore mouillée. Elle est froide, et un peu piquante. Tes chaussures restent dans l'allée, d'accord ? D'accord, maman. Sarah pose les chaussures sur les cailloux. Tes deux pieds sont sur les cailloux. Un oiseau chante dans le cerisier. Tu as entendu l'oiseau ? Oui, papa. Il est haut. À l'école, je veux poser le soleil. Le soleil en papier. Il est dans le cartable. On part. Tu dis au revoir au jardin. Au revoir, jardin. La classe sent les feutres et le papier. La maîtresse parle du temps. Aujourd'hui, il y a du soleil. Bonjour, maîtresse. Sarah écoute. Elle prend le rond jaune, tout léger. Elle pose le soleil sur le tableau. Le papier est lisse. Il tient avec une pince. Merci, Sarah. Plus tard, c'est la sortie. La cour est chaude. Des voix jouent au loin. Près du portail, une voix parle trop près. Sarah sent un malaise. Son ventre se serre. Elle reste près du groupe. Elle regarde la maîtresse. Elle se souvient du jardin. Le soir, le linge est rentré. Le jardin est calme. La porte s'ouvre. Te voilà. Tes chaussures ont un peu de poussière. Sarah pose les chaussures dans l'allée. Elle regarde le cerisier. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le jardin tient le linge comme une main ouverte. Un torchon rouge claque, puis se tait. Le vent du matin est tiède. Le portillon fait un petit bruit de fer. Papa accroche une pince en bois. Le torchon rouge fait comme un drapeau. Tu as senti l'herbe, Sarah ? Elle est froide, un peu piquante. Maman plie une serviette chaude de soleil. Les feuilles du cerisier bougent, lentes. Tu as entendu les feuilles ? Oui, papa. Elles parlent tout haut. Près du volet noir, quelque chose brille. Sur le noir lisse, un &lt;emphasis level="moderate"&gt;éclat de tableau&lt;/emphasis&gt; tremble. Il est petit, papa. C'est le soleil sur le volet. Je veux poser le soleil, maintenant ! Celui de la classe, le rond jaune ? Oui, sur le tableau ! Le cartable attend près des chaussures. Les chaussures, dans l'allée ? Oui, maman. Sarah pose les chaussures sur les cailloux. Tes deux pieds sont sur les cailloux ? Oui. En ce moment, Sarah prend le rond jaune. Le papier est lisse, un peu chaud. Il sent le soleil, maman. On dit au revoir au jardin ? Au revoir, jardin. Le portillon cliquette derrière eux. La classe sent les feutres et le papier. Un carré de soleil glisse sur le tableau. La maîtresse parle près du noir. Bonjour les enfants. Bonjour, maîtresse. Le rond jaune va sur le tableau. Sarah pose le soleil, sans se presser. Le papier tient. Sous le rond, l'éclat de tableau brille. Il est là. Plus tard, c'est la sortie. La cour est chaude. Des voix jouent, plus loin. Près du portail, une voix parle trop près. Sarah sent un malaise. Son ventre se serre, tout petit. Elle reste près du groupe. Elle pense au jardin, au volet. Le soir, le linge est rentré. Le jardin est calme. La porte s'ouvre. Te voilà. Tes chaussures ont un peu de poussière. Sarah veut le dire, tout de suite. Papa, au portail ! Papa parle à maman, près des chaussures. Les mots de Sarah se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Sarah ? Mon ventre s'est serré. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa s'accroupit à sa hauteur. Tu as faim ? Sarah ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Loïc est à l'école. La maîtresse parle du temps. Loïc aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : aujourd'hui, il y a du soleil. Loïc écoute. Il pose le soleil sur le tableau. Plus tard, c'est la sortie. Un adulte près du portail parle tout près. Loïc sent un malaise. Son ventre est serré. Parce qu'il a un malaise, il se souvient. Le soir, papa l'attend. Loïc vient raconter à la maison. Il dit : papa, j'ai eu un malaise au portail. Papa l'écoute. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. Parce qu'il a raconté à la maison, Loïc se sent plus léger. Papa lui tient la main. [pause]</t>
+          <t>Le jardin tient le linge comme une main ouverte. Un torchon rouge claque, puis se tait. Le vent du matin est tiède. Le portillon fait un petit bruit de fer. Papa accroche une pince en bois. Le torchon rouge fait comme un drapeau. Tu as senti l'herbe, Sarah ? Elle est froide, un peu piquante. Maman plie une serviette chaude de soleil. Les feuilles du cerisier bougent, lentes. Tu as entendu les feuilles ? Oui, papa. Elles parlent tout haut. Près du volet noir, quelque chose brille. Sur le noir lisse, un &lt;emphasis&gt;éclat de tableau&lt;/emphasis&gt; tremble. Il est petit, papa. C'est le soleil sur le volet. Je veux poser le soleil, maintenant ! Celui de la classe, le rond jaune ? Oui, sur le tableau ! Le cartable attend près des chaussures. Les chaussures, dans l'allée ? Oui, maman. Sarah pose les chaussures sur les cailloux. Tes deux pieds sont sur les cailloux ? Oui. En ce moment, Sarah prend le rond jaune. Le papier est lisse, un peu chaud. Il sent le soleil, maman. On dit au revoir au jardin ? Au revoir, jardin. Le portillon cliquette derrière eux. La classe sent les feutres et le papier. Un carré de soleil glisse sur le tableau. La maîtresse parle près du noir. Bonjour les enfants. Bonjour, maîtresse. Le rond jaune va sur le tableau. Sarah pose le soleil, sans se presser. Le papier tient. Sous le rond, l'éclat de tableau brille. Il est là. Plus tard, c'est la sortie. La cour est chaude. Des voix jouent, plus loin. Près du portail, une voix parle trop près. Sarah sent un malaise. Son ventre se serre, tout petit. Elle reste près du groupe. Elle pense au jardin, au volet. Le soir, le linge est rentré. Le jardin est calme. La porte s'ouvre. Te voilà. Tes chaussures ont un peu de poussière. Sarah veut le dire, tout de suite. Papa, au portail ! Papa parle à maman, près des chaussures. Les mots de Sarah se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Sarah ? Mon ventre s'est serré. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa s'accroupit à sa hauteur. Tu as faim ? Sarah ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de tableau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,65 +1321,87 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_dire_le_malaise_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le linge danse sur la corde du jardin.
-narrateur|Un torchon rouge claque un peu, tout léger.
+          <t>narrateur|Le jardin tient le linge comme une main ouverte.
+narrateur|Un torchon rouge claque, puis se tait.
 narrateur|Le vent du matin est tiède.
 narrateur|Le portillon fait un petit bruit de fer.
 narrateur|Papa accroche une pince en bois.
-narrateur|Maman plie une serviette encore chaude de soleil.
 papa|Le torchon rouge fait comme un drapeau.
 maman|Tu as senti l'herbe, Sarah ?
-narrateur|En ce moment, Sarah sent l'herbe encore mouillée.
-enfant-f|Elle est froide, et un peu piquante.
-maman|Tes chaussures restent dans l'allée, d'accord ?
-enfant-f|D'accord, maman.
+enfant-f|Elle est froide, un peu piquante.
+narrateur|Maman plie une serviette chaude de soleil.
+narrateur|Les feuilles du cerisier bougent, lentes.
+papa|Tu as entendu les feuilles ?
+enfant-f|Oui, papa.
+enfant-f|Elles parlent tout haut.
+narrateur|Près du volet noir, quelque chose brille.
+narrateur|Sur le noir lisse, un éclat de tableau tremble.
+enfant-f|Il est petit, papa.
+papa|C'est le soleil sur le volet.
+enfant-f|Je veux poser le soleil, maintenant !
+maman|Celui de la classe, le rond jaune ?
+enfant-f|Oui, sur le tableau !
+narrateur|Le cartable attend près des chaussures.
+maman|Les chaussures, dans l'allée ?
+enfant-f|Oui, maman.
 narrateur|Sarah pose les chaussures sur les cailloux.
-papa|Tes deux pieds sont sur les cailloux.
-narrateur|Un oiseau chante dans le cerisier.
-papa|Tu as entendu l'oiseau ?
-enfant-f|Oui, papa.
-enfant-f|Il est haut.
-enfant-f|À l'école, je veux poser le soleil.
-enfant-f|Le soleil en papier.
-maman|Il est dans le cartable.
-maman|On part.
-maman|Tu dis au revoir au jardin.
+papa|Tes deux pieds sont sur les cailloux ?
+enfant-f|Oui.
+narrateur|En ce moment, Sarah prend le rond jaune.
+narrateur|Le papier est lisse, un peu chaud.
+enfant-f|Il sent le soleil, maman.
+maman|On dit au revoir au jardin ?
 enfant-f|Au revoir, jardin.
+narrateur|Le portillon cliquette derrière eux.
 narrateur|La classe sent les feutres et le papier.
-narrateur|La maîtresse parle du temps.
-maitresse|Aujourd'hui, il y a du soleil.
+narrateur|Un carré de soleil glisse sur le tableau.
+narrateur|La maîtresse parle près du noir.
+maitresse|Bonjour les enfants.
 enfant-f|Bonjour, maîtresse.
-narrateur|Sarah écoute.
-narrateur|Elle prend le rond jaune, tout léger.
-narrateur|Elle pose le soleil sur le tableau.
-narrateur|Le papier est lisse.
-narrateur|Il tient avec une pince.
-maitresse|Merci, Sarah.
+maitresse|Le rond jaune va sur le tableau.
+narrateur|Sarah pose le soleil, sans se presser.
+narrateur|Le papier tient.
+narrateur|Sous le rond, l'éclat de tableau brille.
+enfant-f|Il est là.
 narrateur|Plus tard, c'est la sortie.
 narrateur|La cour est chaude.
-narrateur|Des voix jouent au loin.
+narrateur|Des voix jouent, plus loin.
 narrateur|Près du portail, une voix parle trop près.
 narrateur|Sarah sent un malaise.
-narrateur|Son ventre se serre.
+narrateur|Son ventre se serre, tout petit.
 narrateur|Elle reste près du groupe.
-narrateur|Elle regarde la maîtresse.
-narrateur|Elle se souvient du jardin.
+narrateur|Elle pense au jardin, au volet.
 narrateur|Le soir, le linge est rentré.
 narrateur|Le jardin est calme.
 narrateur|La porte s'ouvre.
 papa|Te voilà.
 papa|Tes chaussures ont un peu de poussière.
-narrateur|Sarah pose les chaussures dans l'allée.
-narrateur|Elle regarde le cerisier.
-narrateur|Le ventre est encore serré.</t>
+narrateur|Sarah veut le dire, tout de suite.
+enfant-f|Papa, au portail !
+narrateur|Papa parle à maman, près des chaussures.
+narrateur|Les mots de Sarah se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Sarah ?
+enfant-f|Mon ventre s'est serré.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Ça ne sort pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à sa hauteur.
+papa|Tu as faim ?
+narrateur|Sarah ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc,porte</t>
+          <t>linge,portillon</t>
         </is>
       </c>
     </row>
@@ -1411,22 +1433,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah a un malaise. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Loïc a un malaise. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>elle raconte</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>écouter | raconter | à la maison | papa | malaise</t>
+          <t>elle raconte | raconter | au goûter | au gouter | à papa | à la maison | elle attend | elle dit | papa | malaise</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1441,7 +1463,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle écoute la maîtresse. Puis elle raconte à la maison. Que fait Sarah ?</t>
+          <t>Sarah a un malaise. Elle raconte au goûter. Que fait-elle ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1479,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1490,7 +1512,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1505,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1547,17 +1573,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_raconte_au_gouter; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1590,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa. J'ai eu un malaise au portail. On t'écoute. Viens près de la fenêtre. Sarah parle, tout bas. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Sarah se sent plus légère. Le torchon rouge repose, plié.</t>
+          <t>Sarah ouvre la bouche trop vite. Papa, au portail, quelqu'un parlait ! Papa n'a pas fini sa phrase. Les chaussures, dans l'allée, Sarah. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la maison, un instant. Le goûter est près de la fenêtre. Papa pose un verre d'eau. Maman pose une pêche. Sarah attend que le silence arrive. Sur le volet, l'éclat de tableau brille. Je peux te dire quelque chose ? Oui, nous t'écoutons. Au portail, quelqu'un a parlé trop près. Mon ventre s'est serré. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Papa. J'ai eu un malaise au portail. On t'écoute. Viens près de la fenêtre. Sarah parle, tout bas. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Sarah se sent plus légère. Le torchon rouge repose, plié.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah ouvre la bouche trop vite. Papa, au portail, quelqu'un parlait ! Papa n'a pas fini sa phrase. Les chaussures, dans l'allée, Sarah. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la maison, un instant. Le &lt;emphasis level="moderate"&gt;goûter&lt;/emphasis&gt; est près de la fenêtre. Papa pose un verre d'eau. Maman pose une pêche. Sarah attend que le silence arrive. Sur le volet, l'éclat de tableau brille. Je peux te dire quelque chose ? Oui, nous t'écoutons. Au portail, quelqu'un a parlé trop près. Mon ventre s'est serré. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Loïc a écouté. Il a raconté son malaise à la maison. Papa est là. [pause]</t>
+          <t>Sarah ouvre la bouche trop vite. Papa, au portail, quelqu'un parlait ! Papa n'a pas fini sa phrase. Les chaussures, dans l'allée, Sarah. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la maison, un instant. Le &lt;emphasis&gt;goûter&lt;/emphasis&gt; est près de la fenêtre. Papa pose un verre d'eau. Maman pose une pêche. Sarah attend que le silence arrive. Sur le volet, l'éclat de tableau brille. Je peux te dire quelque chose ? Oui, nous t'écoutons. Au portail, quelqu'un a parlé trop près. Mon ventre s'est serré. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1658,7 +1684,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,9 +1705,13 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>goûter</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>450</v>
@@ -1691,16 +1721,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1725,23 +1755,41 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=elle_refuse_de_foncer_puis_raconte; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Papa.
-enfant-f|J'ai eu un malaise au portail.
-papa|On t'écoute.
-maman|Viens près de la fenêtre.
-narrateur|Sarah parle, tout bas.
-narrateur|Papa écoute.
-narrateur|Maman écoute.
-papa|Tu as bien fait de raconter.
-maman|À l'école, on écoute la maîtresse.
-papa|Si tu as un malaise, tu viens le dire.
-narrateur|Sarah se sent plus légère.
-narrateur|Le torchon rouge repose, plié.</t>
+          <t>narrateur|Sarah ouvre la bouche trop vite.
+enfant-f|Papa, au portail, quelqu'un parlait !
+narrateur|Papa n'a pas fini sa phrase.
+papa|Les chaussures, dans l'allée, Sarah.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle pose les mains à plat.
+narrateur|Elle écoute la maison, un instant.
+maman|Le goûter est près de la fenêtre.
+narrateur|Papa pose un verre d'eau.
+narrateur|Maman pose une pêche.
+narrateur|Sarah attend que le silence arrive.
+narrateur|Sur le volet, l'éclat de tableau brille.
+enfant-f|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-f|Au portail, quelqu'un a parlé trop près.
+enfant-f|Mon ventre s'est serré.
+papa|Merci, Sarah.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as soif ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Sarah se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>peche,verre</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah range son cartable près de la porte. Papa prépare le goûter. Une pêche, un peu d'eau. Tu t'assois près de la fenêtre ? Oui. On voit le cerisier. Tes pieds sont sur le tapis. Sarah croque la pêche. Elle est sucrée. Le vrai soleil est sur le cerisier. Et le papier était sur le tableau. Oui. Il tenait avec la pince. Le jardin sent l'herbe sèche. Le vent s'est calmé. Merci, papa. Merci, maman.</t>
+          <t>Sarah range son cartable près de la porte. On s'assoit près de la fenêtre ? Oui. On voit le cerisier. La pêche est sucrée, un peu chaude. Le jardin sent l'herbe sèche. Tes pieds sont sur le tapis ? Oui, maman. Sarah veut raconter la cour, d'un coup. Les mots se bousculent dans sa bouche. Attends. Elle refuse de foncer. Elle reprend, plus lentement. La cour était chaude. J'ai posé le soleil. Le rond jaune, sur le tableau ? Oui, et l'éclat était là. Sarah croque la pêche. Un peu de jus reste sur le doigt. Il est sucré ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah range son cartable près de la porte. Papa prépare le goûter. Une pêche, un peu d'eau. Tu t'assois près de la fenêtre ? Oui. On voit le cerisier. Tes pieds sont sur le tapis. Sarah croque la pêche. Elle est sucrée. Le vrai soleil est sur le cerisier. Et le papier était sur le tableau. Oui. Il tenait avec la pince. Le jardin sent l'herbe sèche. Le vent s'est calmé. Merci, papa. Merci, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah range son cartable près de la porte. On s'assoit près de la fenêtre ? Oui. On voit le cerisier. La pêche est sucrée, un peu chaude. Le jardin sent l'herbe sèche. Tes pieds sont sur le tapis ? Oui, maman. Sarah veut raconter la cour, d'un coup. Les mots se bousculent dans sa bouche. Attends. Elle refuse de foncer. Elle reprend, plus lentement. La cour était chaude. J'ai posé le soleil. Le rond jaune, sur le tableau ? Oui, et l'éclat était là. Sarah croque la pêche. Un peu de jus reste sur le doigt. Il est sucré ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Loïc range son cartable. Papa prépare le goûter. [pause]</t>
+          <t>Sarah range son cartable près de la porte. On s'assoit près de la fenêtre ? Oui. On voit le cerisier. La pêche est sucrée, un peu chaude. Le jardin sent l'herbe sèche. Tes pieds sont sur le tapis ? Oui, maman. Sarah veut raconter la cour, d'un coup. Les mots se bousculent dans sa bouche. Attends. Elle refuse de foncer. Elle reprend, plus lentement. La cour était chaude. J'ai posé le soleil. Le rond jaune, sur le tableau ? Oui, et l'éclat était là. Sarah croque la pêche. Un peu de jus reste sur le doigt. Il est sucré ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1833,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1859,26 +1907,26 @@
       </c>
       <c r="AH5" s="2" t="inlineStr"/>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,10 +1935,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1901,26 +1949,39 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_eclat_tient; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Sarah range son cartable près de la porte.
-narrateur|Papa prépare le goûter.
-narrateur|Une pêche, un peu d'eau.
-maman|Tu t'assois près de la fenêtre ?
+papa|On s'assoit près de la fenêtre ?
 enfant-f|Oui.
-enfant-f|On voit le cerisier.
-papa|Tes pieds sont sur le tapis.
+narrateur|On voit le cerisier.
+narrateur|La pêche est sucrée, un peu chaude.
+enfant-f|Le jardin sent l'herbe sèche.
+maman|Tes pieds sont sur le tapis ?
+enfant-f|Oui, maman.
+narrateur|Sarah veut raconter la cour, d'un coup.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Attends.
+narrateur|Elle refuse de foncer.
+narrateur|Elle reprend, plus lentement.
+enfant-f|La cour était chaude.
+enfant-f|J'ai posé le soleil.
+papa|Le rond jaune, sur le tableau ?
+enfant-f|Oui, et l'éclat était là.
 narrateur|Sarah croque la pêche.
-narrateur|Elle est sucrée.
-enfant-f|Le vrai soleil est sur le cerisier.
-maman|Et le papier était sur le tableau.
-enfant-f|Oui.
-enfant-f|Il tenait avec la pince.
-narrateur|Le jardin sent l'herbe sèche.
-narrateur|Le vent s'est calmé.
-enfant-f|Merci, papa.
-enfant-f|Merci, maman.</t>
+narrateur|Un peu de jus reste sur le doigt.
+maman|Il est sucré ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>peche,fenetre</t>
         </is>
       </c>
     </row>
@@ -1947,17 +2008,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le torchon rouge dort dans le panier. Le cerisier garde un peu de soleil. On t'a écoutée, Sarah. Tu as posé le soleil.</t>
+          <t>Le torchon rouge est rentré. Il est plié, près de la porte. Le volet noir garde un peu de soleil. Comme sur le tableau, papa ! Tu le vois, toi ? Oui, sur le noir. Le vent tiède pousse une feuille du cerisier. On est bien, ici. La pêche est finie ? Presque, maman. Sarah pose le noyau dans la coupelle. L'éclat de tableau tient sur le volet.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le torchon rouge dort dans le panier. Le cerisier garde un peu de soleil. On t'a écoutée, Sarah. Tu as posé le soleil.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le torchon rouge est rentré. Il est plié, près de la porte. Le volet noir garde un peu de soleil. Comme sur le tableau, papa ! Tu le vois, toi ? Oui, sur le noir. Le vent tiède pousse une feuille du cerisier. On est bien, ici. La pêche est finie ? Presque, maman. Sarah pose le noyau dans la coupelle. L'&lt;emphasis level="moderate"&gt;éclat de tableau&lt;/emphasis&gt; tient sur le volet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le torchon rouge est rentré. Il est plié, près de la porte. Le volet noir garde un peu de soleil. Comme sur le tableau, papa ! Tu le vois, toi ? Oui, sur le noir. Le vent tiède pousse une feuille du cerisier. On est bien, ici. La pêche est finie ? Presque, maman. Sarah pose le noyau dans la coupelle. L'&lt;emphasis&gt;éclat de tableau&lt;/emphasis&gt; tient sur le volet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2004,7 +2065,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2012,10 +2073,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2024,12 +2085,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2038,17 +2099,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tableau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2057,11 +2122,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2070,27 +2135,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_tient_sur_le_volet; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le torchon rouge dort dans le panier.
-narrateur|Le cerisier garde un peu de soleil.
-papa|On t'a écoutée, Sarah.
-maman|Tu as posé le soleil.</t>
+          <t>enfant-f|Le torchon rouge est rentré.
+maman|Il est plié, près de la porte.
+narrateur|Le volet noir garde un peu de soleil.
+enfant-f|Comme sur le tableau, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le noir.
+narrateur|Le vent tiède pousse une feuille du cerisier.
+enfant-f|On est bien, ici.
+maman|La pêche est finie ?
+enfant-f|Presque, maman.
+narrateur|Sarah pose le noyau dans la coupelle.
+narrateur|L'éclat de tableau tient sur le volet.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>vent,cerisier</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2168,6 +2250,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>